<commit_message>
added some dummy data for presentation purposes
</commit_message>
<xml_diff>
--- a/demand_max.xlsx
+++ b/demand_max.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uzk-my.sharepoint.com/personal/linus_palm_uzk_onmicrosoft_com/Documents/Master/MA/master-thesis-nurse-scheduling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{7C85814F-0396-AB4C-876E-7801D68A3AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE2A104E-E1D0-A643-B827-15349FCD1CF5}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="13_ncr:1_{7C85814F-0396-AB4C-876E-7801D68A3AEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93D6635A-0A4B-3943-9ACB-76896B0122A2}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" xr2:uid="{F6C4B857-2221-7442-B2F7-99991C74024F}"/>
   </bookViews>
@@ -130,6 +130,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -449,10 +453,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5726D70-3220-EE45-8CC4-80523B43DD04}">
-  <dimension ref="A1:AF4"/>
+  <dimension ref="A1:AE4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -546,11 +550,8 @@
       <c r="AE1" s="1">
         <v>29</v>
       </c>
-      <c r="AF1" s="1">
-        <v>30</v>
-      </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -644,11 +645,8 @@
       <c r="AE2" s="2">
         <v>5</v>
       </c>
-      <c r="AF2" s="2">
-        <v>5</v>
-      </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -742,11 +740,8 @@
       <c r="AE3" s="2">
         <v>4</v>
       </c>
-      <c r="AF3" s="2">
-        <v>4</v>
-      </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -838,9 +833,6 @@
         <v>3</v>
       </c>
       <c r="AE4" s="2">
-        <v>3</v>
-      </c>
-      <c r="AF4" s="2">
         <v>3</v>
       </c>
     </row>

</xml_diff>